<commit_message>
docs: enrich README.md with comprehensive 5-component COGS, investor-grade decision note and sensitivity analysis
</commit_message>
<xml_diff>
--- a/2A202601063_NguyenDucAnh_Day24.xlsx
+++ b/2A202601063_NguyenDucAnh_Day24.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\aaaaaa\Track1_Day24_NguyenDucAnh_2A202601063\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4123E07A-3BE0-46CB-9E70-2F66ECAB705A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B703CF42-9504-4494-A755-DD5C19FB0E39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -847,7 +847,7 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -1935,7 +1935,7 @@
       <c r="E38" s="50"/>
       <c r="F38" s="50"/>
     </row>
-    <row r="39" spans="2:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:7" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="53" t="s">
         <v>51</v>
       </c>
@@ -1944,14 +1944,14 @@
       <c r="E39" s="54"/>
       <c r="F39" s="54"/>
     </row>
-    <row r="40" spans="2:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:7" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="55"/>
       <c r="C40" s="50"/>
       <c r="D40" s="50"/>
       <c r="E40" s="50"/>
       <c r="F40" s="50"/>
     </row>
-    <row r="41" spans="2:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:7" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="55"/>
       <c r="C41" s="50"/>
       <c r="D41" s="50"/>
@@ -1960,7 +1960,8 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="B34:F34"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="B39:F41"/>
@@ -1969,8 +1970,7 @@
     <mergeCell ref="B30:F30"/>
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="B24:F24"/>
-    <mergeCell ref="B38:F38"/>
-    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="B2:F2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>